<commit_message>
[Doc][FD]The fault type Excel file is updated
Co-authored-by: liujp20<305870551@qq.com>
</commit_message>
<xml_diff>
--- a/docs/zh/resource/故障诊断类型.xlsx
+++ b/docs/zh/resource/故障诊断类型.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="根因设备分析故障事件" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="网络拥塞分析故障事件" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="设备资源分析故障事件" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="根因节点分析故障场景" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="根因设备分析故障事件" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="网络拥塞分析故障事件" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="设备资源分析故障事件" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="根因节点分析故障场景" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1093"/>
+  <dimension ref="A1:G1094"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -40269,12 +40269,12 @@
       </c>
       <c r="E1067" s="2" t="inlineStr">
         <is>
-          <t>tp中psn配置错误</t>
+          <t>疑似tp中psn配置错误</t>
         </is>
       </c>
       <c r="F1067" s="2" t="inlineStr">
         <is>
-          <t>内核日志上报了"udma....ae....event type is 2....sub type is 3"描述且twp_ae_dfx指标值对应二进制第3位为1，表示tp中psn配置错误</t>
+          <t>内核日志上报了"udma....ae....event type is 2....sub type is 3"描述且twp_ae_dfx指标值对应二进制第3位为1，疑似tp中psn配置错误</t>
         </is>
       </c>
       <c r="G1067" s="2" t="inlineStr">
@@ -40346,12 +40346,12 @@
       </c>
       <c r="E1069" s="2" t="inlineStr">
         <is>
-          <t>ctp的拥塞为关闭</t>
+          <t>ctp的拥塞未关闭</t>
         </is>
       </c>
       <c r="F1069" s="2" t="inlineStr">
         <is>
-          <t>tain_compact_top_alarm指标值对应二进制第6位为1，表示ctp的拥塞为关闭</t>
+          <t>tai_compact_top_alarm指标值对应二进制第6位为1，表示ctp的拥塞未关闭</t>
         </is>
       </c>
       <c r="G1069" s="2" t="inlineStr">
@@ -40891,39 +40891,39 @@
       </c>
       <c r="C1084" s="2" t="inlineStr">
         <is>
-          <t>UB</t>
+          <t>RDMA</t>
         </is>
       </c>
       <c r="D1084" s="2" t="inlineStr">
         <is>
-          <t>Comp_CANN_HCCL_Custom_CQE0x5</t>
+          <t>Comp_Custom_CQE0x5_RXDMA_ICRC_ERR</t>
         </is>
       </c>
       <c r="E1084" s="2" t="inlineStr">
         <is>
-          <t>软件故障</t>
+          <t>RX DMA ICRC错误计数增长</t>
         </is>
       </c>
       <c r="F1084" s="2" t="inlineStr">
         <is>
-          <t>无RAS告警且HCCL通信上报CQE ERROR 0x5</t>
+          <t>任务前后对比，hccn_tool工具查询端口的相关统计信息中rxdma_icrc_err_cnt_queue_id{0~3}任一计数出现增长（after &gt; before），链路存在ICRC错误</t>
         </is>
       </c>
       <c r="G1084" s="2" t="inlineStr">
         <is>
-          <t>['收集NPU日志，联系华为工程师进一步定位详细根因']</t>
+          <t>['通过hccl-test工具校验数据，结合链路二分排查对应的故障芯片位置。']</t>
         </is>
       </c>
     </row>
     <row r="1085">
       <c r="A1085" s="2" t="inlineStr">
         <is>
-          <t>Hardware</t>
+          <t>Software</t>
         </is>
       </c>
       <c r="B1085" s="2" t="inlineStr">
         <is>
-          <t>UB Switch</t>
+          <t>NPU</t>
         </is>
       </c>
       <c r="C1085" s="2" t="inlineStr">
@@ -40933,22 +40933,22 @@
       </c>
       <c r="D1085" s="2" t="inlineStr">
         <is>
-          <t>0x08520006</t>
+          <t>Comp_CANN_HCCL_Custom_CQE0x5</t>
         </is>
       </c>
       <c r="E1085" s="2" t="inlineStr">
         <is>
-          <t>接口状态为ERROR DOWN</t>
+          <t>软件故障</t>
         </is>
       </c>
       <c r="F1085" s="2" t="inlineStr">
         <is>
-          <t>具体报错原因可根据故障原始信息中"Cause="的值，结合文档"https://support.huawei.com/enterprise/zh/doc/EDOC1100591431/aa27ae3b?idPath=23710424|251366513|22892968|263594706#ZH-CN_ALARMREF_0000002601566845"进行定位</t>
+          <t>无RAS告警且HCCL通信上报CQE ERROR 0x5</t>
         </is>
       </c>
       <c r="G1085" s="2" t="inlineStr">
         <is>
-          <t>['在查找报错原因的文档中按照对应原因的处理建议进行操作']</t>
+          <t>['收集NPU日志，联系华为工程师进一步定位详细根因']</t>
         </is>
       </c>
     </row>
@@ -40970,22 +40970,22 @@
       </c>
       <c r="D1086" s="2" t="inlineStr">
         <is>
-          <t>0x081320C6</t>
+          <t>0x08520006</t>
         </is>
       </c>
       <c r="E1086" s="2" t="inlineStr">
         <is>
-          <t>本端接口故障</t>
+          <t>接口状态为ERROR DOWN</t>
         </is>
       </c>
       <c r="F1086" s="2" t="inlineStr">
         <is>
-          <t>远端接口到本端接口之间链路产生故障，如接收光纤瞬断、本端接口所在子卡故障或光模块异常等</t>
+          <t>具体报错原因可根据故障原始信息中"Cause="的值，结合文档"https://support.huawei.com/enterprise/zh/doc/EDOC1100591431/aa27ae3b?idPath=23710424|251366513|22892968|263594706#ZH-CN_ALARMREF_0000002601566845"进行定位</t>
         </is>
       </c>
       <c r="G1086" s="2" t="inlineStr">
         <is>
-          <t>['1. 检查发送光纤是否故障。\n如果是，请更换光纤。\n如果不是，请执行步骤2。\n2. 检查本端接口和远端接口的光模块是否故障。\n如果是，请更换光模块。\n如果不是，请执行步骤3。\n3. 检查本端设备和远端设备单板是否故障。\n如果是，请更换单板。\n如果不是，请执行步骤4。\n4. 请收集告警信息、日志信息和配置信息，并联系技术支持人员。']</t>
+          <t>['在查找报错原因的文档中按照对应原因的处理建议进行操作']</t>
         </is>
       </c>
     </row>
@@ -41007,22 +41007,22 @@
       </c>
       <c r="D1087" s="2" t="inlineStr">
         <is>
-          <t>0x081320C7</t>
+          <t>0x081320C6</t>
         </is>
       </c>
       <c r="E1087" s="2" t="inlineStr">
         <is>
-          <t>远端故障告警</t>
+          <t>本端接口故障</t>
         </is>
       </c>
       <c r="F1087" s="2" t="inlineStr">
         <is>
-          <t>本端到远端的发送链路产生故障，例如拔掉本端的发送光纤，导致远端无法接收，则本端（仅支持10GE以上速率端口的设备）会上报该告警。</t>
+          <t>远端接口到本端接口之间链路产生故障，如接收光纤瞬断、本端接口所在子卡故障或光模块异常等</t>
         </is>
       </c>
       <c r="G1087" s="2" t="inlineStr">
         <is>
-          <t>['1.检查发送光纤是否故障，更换光纤后，检查告警是否恢复。\n如果是，结束。\n如果否，进入步骤2.\n2.检查本端和远端的光模块是否故障，更换光模块后，检查告警是否恢复。\n如果是，结束。\n如果否，进入步骤3.\n3.检查远端单板是否故障，更换单板后，检查告警是否恢复。\n如果是，结束。\n如果否，进入步骤4.\n4.请收集告警信息、日志信息和配置信息，联系华为工程师进行处理。']</t>
+          <t>['1. 检查发送光纤是否故障。\n如果是，请更换光纤。\n如果不是，请执行步骤2。\n2. 检查本端接口和远端接口的光模块是否故障。\n如果是，请更换光模块。\n如果不是，请执行步骤3。\n3. 检查本端设备和远端设备单板是否故障。\n如果是，请更换单板。\n如果不是，请执行步骤4。\n4. 请收集告警信息、日志信息和配置信息，并联系技术支持人员。']</t>
         </is>
       </c>
     </row>
@@ -41044,22 +41044,22 @@
       </c>
       <c r="D1088" s="2" t="inlineStr">
         <is>
-          <t>0x08132247</t>
+          <t>0x081320C7</t>
         </is>
       </c>
       <c r="E1088" s="2" t="inlineStr">
         <is>
-          <t>电口SNR值异常，网线质量差</t>
+          <t>远端故障告警</t>
         </is>
       </c>
       <c r="F1088" s="2" t="inlineStr">
         <is>
-          <t>网线质量不好或存在信号干扰</t>
+          <t>本端到远端的发送链路产生故障，例如拔掉本端的发送光纤，导致远端无法接收，则本端（仅支持10GE以上速率端口的设备）会上报该告警。</t>
         </is>
       </c>
       <c r="G1088" s="2" t="inlineStr">
         <is>
-          <t>['1.更换高质量网线，如Cat6A网线或屏蔽网线。', '2.降低电口的工作速率。', '3.请联系技术支持人员。']</t>
+          <t>['1.检查发送光纤是否故障，更换光纤后，检查告警是否恢复。\n如果是，结束。\n如果否，进入步骤2.\n2.检查本端和远端的光模块是否故障，更换光模块后，检查告警是否恢复。\n如果是，结束。\n如果否，进入步骤3.\n3.检查远端单板是否故障，更换单板后，检查告警是否恢复。\n如果是，结束。\n如果否，进入步骤4.\n4.请收集告警信息、日志信息和配置信息，联系华为工程师进行处理。']</t>
         </is>
       </c>
     </row>
@@ -41081,22 +41081,22 @@
       </c>
       <c r="D1089" s="2" t="inlineStr">
         <is>
-          <t>0x08130054</t>
+          <t>0x08132247</t>
         </is>
       </c>
       <c r="E1089" s="2" t="inlineStr">
         <is>
-          <t>单板局部功能失效</t>
+          <t>电口SNR值异常，网线质量差</t>
         </is>
       </c>
       <c r="F1089" s="2" t="inlineStr">
         <is>
-          <t>具体报错原因可根据故障原始信息中"Reason="的值，结合文档"https://support.huawei.com/enterprise/zh/doc/EDOC1100591431/5f604ea7?idPath=23710424|251366513|22892968|263594706"进行定位</t>
+          <t>网线质量不好或存在信号干扰</t>
         </is>
       </c>
       <c r="G1089" s="2" t="inlineStr">
         <is>
-          <t>['在查找报错原因的文档中按照对应原因的处理建议进行操作']</t>
+          <t>['1.更换高质量网线，如Cat6A网线或屏蔽网线。', '2.降低电口的工作速率。', '3.请联系技术支持人员。']</t>
         </is>
       </c>
     </row>
@@ -41118,17 +41118,17 @@
       </c>
       <c r="D1090" s="2" t="inlineStr">
         <is>
-          <t>0x0813002E</t>
+          <t>0x08130054</t>
         </is>
       </c>
       <c r="E1090" s="2" t="inlineStr">
         <is>
-          <t>单板整体功能失效</t>
+          <t>单板局部功能失效</t>
         </is>
       </c>
       <c r="F1090" s="2" t="inlineStr">
         <is>
-          <t>具体报错原因可根据故障原始信息中"Reason="的值，结合文档"https://support.huawei.com/enterprise/zh/doc/EDOC1100591431/fb46a5c6?idPath=23710424|251366513|22892968|263594706"进行定位</t>
+          <t>具体报错原因可根据故障原始信息中"Reason="的值，结合文档"https://support.huawei.com/enterprise/zh/doc/EDOC1100591431/5f604ea7?idPath=23710424|251366513|22892968|263594706"进行定位</t>
         </is>
       </c>
       <c r="G1090" s="2" t="inlineStr">
@@ -41155,61 +41155,61 @@
       </c>
       <c r="D1091" s="2" t="inlineStr">
         <is>
+          <t>0x0813002E</t>
+        </is>
+      </c>
+      <c r="E1091" s="2" t="inlineStr">
+        <is>
+          <t>单板整体功能失效</t>
+        </is>
+      </c>
+      <c r="F1091" s="2" t="inlineStr">
+        <is>
+          <t>具体报错原因可根据故障原始信息中"Reason="的值，结合文档"https://support.huawei.com/enterprise/zh/doc/EDOC1100591431/fb46a5c6?idPath=23710424|251366513|22892968|263594706"进行定位</t>
+        </is>
+      </c>
+      <c r="G1091" s="2" t="inlineStr">
+        <is>
+          <t>['在查找报错原因的文档中按照对应原因的处理建议进行操作']</t>
+        </is>
+      </c>
+    </row>
+    <row r="1092">
+      <c r="A1092" s="2" t="inlineStr">
+        <is>
+          <t>Hardware</t>
+        </is>
+      </c>
+      <c r="B1092" s="2" t="inlineStr">
+        <is>
+          <t>UB Switch</t>
+        </is>
+      </c>
+      <c r="C1092" s="2" t="inlineStr">
+        <is>
+          <t>UB</t>
+        </is>
+      </c>
+      <c r="D1092" s="2" t="inlineStr">
+        <is>
           <t>0x08130056</t>
         </is>
       </c>
-      <c r="E1091" s="2" t="inlineStr">
+      <c r="E1092" s="2" t="inlineStr">
         <is>
           <t>子卡局部功能失效</t>
         </is>
       </c>
-      <c r="F1091" s="2" t="inlineStr">
+      <c r="F1092" s="2" t="inlineStr">
         <is>
           <t>原因1：Failed to check the voltage of the card.（子卡电压检查失败）
 原因2：The sensor on the subcard was faulty.（子卡传感器故障。）
 原因3：The soft-start mos was over temperature.（软启动mos温度过高。）</t>
         </is>
       </c>
-      <c r="G1091" s="2" t="inlineStr">
+      <c r="G1092" s="2" t="inlineStr">
         <is>
           <t>['请收集告警信息、日志信息和配置信息，并联系技术支持人员。']</t>
-        </is>
-      </c>
-    </row>
-    <row r="1092">
-      <c r="A1092" s="2" t="inlineStr">
-        <is>
-          <t>Hardware</t>
-        </is>
-      </c>
-      <c r="B1092" s="2" t="inlineStr">
-        <is>
-          <t>UB Switch</t>
-        </is>
-      </c>
-      <c r="C1092" s="2" t="inlineStr">
-        <is>
-          <t>UB</t>
-        </is>
-      </c>
-      <c r="D1092" s="2" t="inlineStr">
-        <is>
-          <t>0x08130059</t>
-        </is>
-      </c>
-      <c r="E1092" s="2" t="inlineStr">
-        <is>
-          <t>光模块异常</t>
-        </is>
-      </c>
-      <c r="F1092" s="2" t="inlineStr">
-        <is>
-          <t>具体报错原因可根据故障原始信息中“Reason=”的值，结合文档“https://support.huawei.com/enterprise/zh/doc/EDOC1100591431/eabd511e?idPath=23710424|251366513|22892968|263594706”进行定位</t>
-        </is>
-      </c>
-      <c r="G1092" s="2" t="inlineStr">
-        <is>
-          <t>['在查找报错原因的文档中按照对应原因的处理建议进行操作']</t>
         </is>
       </c>
     </row>
@@ -41231,20 +41231,57 @@
       </c>
       <c r="D1093" s="2" t="inlineStr">
         <is>
+          <t>0x08130059</t>
+        </is>
+      </c>
+      <c r="E1093" s="2" t="inlineStr">
+        <is>
+          <t>光模块异常</t>
+        </is>
+      </c>
+      <c r="F1093" s="2" t="inlineStr">
+        <is>
+          <t>具体报错原因可根据故障原始信息中“Reason=”的值，结合文档“https://support.huawei.com/enterprise/zh/doc/EDOC1100591431/eabd511e?idPath=23710424|251366513|22892968|263594706”进行定位</t>
+        </is>
+      </c>
+      <c r="G1093" s="2" t="inlineStr">
+        <is>
+          <t>['在查找报错原因的文档中按照对应原因的处理建议进行操作']</t>
+        </is>
+      </c>
+    </row>
+    <row r="1094">
+      <c r="A1094" s="2" t="inlineStr">
+        <is>
+          <t>Hardware</t>
+        </is>
+      </c>
+      <c r="B1094" s="2" t="inlineStr">
+        <is>
+          <t>UB Switch</t>
+        </is>
+      </c>
+      <c r="C1094" s="2" t="inlineStr">
+        <is>
+          <t>UB</t>
+        </is>
+      </c>
+      <c r="D1094" s="2" t="inlineStr">
+        <is>
           <t>0x08520004</t>
         </is>
       </c>
-      <c r="E1093" s="2" t="inlineStr">
+      <c r="E1094" s="2" t="inlineStr">
         <is>
           <t>接口IPv6状态改变</t>
         </is>
       </c>
-      <c r="F1093" s="2" t="inlineStr">
+      <c r="F1094" s="2" t="inlineStr">
         <is>
           <t>具体报错原因可根据故障原始信息中“Reason=”的值，结合文档“https://support.huawei.com/enterprise/zh/doc/EDOC1100591431/2cc877d0?idPath=23710424|251366513|22892968|263594706”进行定位</t>
         </is>
       </c>
-      <c r="G1093" s="2" t="inlineStr">
+      <c r="G1094" s="2" t="inlineStr">
         <is>
           <t>['在查找报错原因的文档中按照对应原因的处理建议进行操作']</t>
         </is>

</xml_diff>